<commit_message>
feat: agregar ambientacion, sonidos y estados finales
</commit_message>
<xml_diff>
--- a/docs/Tareas_Juego_MATE1133.xlsx
+++ b/docs/Tareas_Juego_MATE1133.xlsx
@@ -70,67 +70,67 @@
     <t>xelo</t>
   </si>
   <si>
+    <t>A·sen(Bx+C)+D distinta en cada enemigo, escrita en el código</t>
+  </si>
+  <si>
+    <t>Oleadas 1, 2, 3 y jefe final</t>
+  </si>
+  <si>
+    <t>Oleada 1: tipo 1 · Oleada 2: tipos 1 y 2 · Oleada 3: tipos 1, 2 y 3</t>
+  </si>
+  <si>
+    <t>Munición parabólica con cooldown o cantidad limitada</t>
+  </si>
+  <si>
+    <t>Elegir la orientación de la parábola</t>
+  </si>
+  <si>
+    <t>Enemigo 3 y jefe final: diseño y ecuación propios</t>
+  </si>
+  <si>
+    <t>Diseños distintos en forma, tamaño o estructura, no solo color</t>
+  </si>
+  <si>
+    <t>Munición de otra cónica (elipse, hipérbola o circunferencia)</t>
+  </si>
+  <si>
+    <t>Con cooldown o cantidad limitada</t>
+  </si>
+  <si>
+    <t>Vida de cada enemigo según la munición que lo impacta</t>
+  </si>
+  <si>
+    <t>Las municiones complejas hacen más daño</t>
+  </si>
+  <si>
+    <t>Colisiones, vida de la nave y daño por tipo de enemigo</t>
+  </si>
+  <si>
+    <t>El jefe es el más letal; enemigos no se eliminan entre ellos</t>
+  </si>
+  <si>
+    <t>Integración y balance de daños</t>
+  </si>
+  <si>
+    <t>Los 3</t>
+  </si>
+  <si>
     <t>En revisión</t>
   </si>
   <si>
-    <t>A·sen(Bx+C)+D distinta en cada enemigo, escrita en el código</t>
-  </si>
-  <si>
-    <t>Oleadas 1, 2, 3 y jefe final</t>
-  </si>
-  <si>
-    <t>Oleada 1: tipo 1 · Oleada 2: tipos 1 y 2 · Oleada 3: tipos 1, 2 y 3</t>
-  </si>
-  <si>
-    <t>Munición parabólica con cooldown o cantidad limitada</t>
-  </si>
-  <si>
-    <t>Elegir la orientación de la parábola</t>
-  </si>
-  <si>
-    <t>Enemigo 3 y jefe final: diseño y ecuación propios</t>
-  </si>
-  <si>
-    <t>Diseños distintos en forma, tamaño o estructura, no solo color</t>
-  </si>
-  <si>
-    <t>Munición de otra cónica (elipse, hipérbola o circunferencia)</t>
-  </si>
-  <si>
-    <t>Con cooldown o cantidad limitada</t>
-  </si>
-  <si>
-    <t>Vida de cada enemigo según la munición que lo impacta</t>
+    <t>Jerarquía clara entre enemigos, municiones y jefe</t>
+  </si>
+  <si>
+    <t>Revisión final del código</t>
+  </si>
+  <si>
+    <t>Sin comentarios ni docstrings; solo pygame, math y random; sin errores</t>
+  </si>
+  <si>
+    <t>Eliminar README.md del repositorio</t>
   </si>
   <si>
     <t>Por hacer</t>
-  </si>
-  <si>
-    <t>Las municiones complejas hacen más daño</t>
-  </si>
-  <si>
-    <t>Colisiones, vida de la nave y daño por tipo de enemigo</t>
-  </si>
-  <si>
-    <t>El jefe es el más letal; enemigos no se eliminan entre ellos</t>
-  </si>
-  <si>
-    <t>Integración y balance de daños</t>
-  </si>
-  <si>
-    <t>Los 3</t>
-  </si>
-  <si>
-    <t>Jerarquía clara entre enemigos, municiones y jefe</t>
-  </si>
-  <si>
-    <t>Revisión final del código</t>
-  </si>
-  <si>
-    <t>Sin comentarios ni docstrings; solo pygame, math y random; sin errores</t>
-  </si>
-  <si>
-    <t>Eliminar README.md del repositorio</t>
   </si>
   <si>
     <t>Antes de grabar el video y de entregar</t>
@@ -673,10 +673,10 @@
         <v>46311.0</v>
       </c>
       <c r="E8" s="7" t="s">
+        <v>10</v>
+      </c>
+      <c r="F8" s="5" t="s">
         <v>19</v>
-      </c>
-      <c r="F8" s="5" t="s">
-        <v>20</v>
       </c>
     </row>
     <row r="9" ht="30.0" customHeight="1">
@@ -684,7 +684,7 @@
         <v>5.0</v>
       </c>
       <c r="B9" s="5" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="C9" s="4" t="s">
         <v>9</v>
@@ -696,7 +696,7 @@
         <v>10</v>
       </c>
       <c r="F9" s="5" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
     </row>
     <row r="10" ht="30.0" customHeight="1">
@@ -704,7 +704,7 @@
         <v>6.0</v>
       </c>
       <c r="B10" s="5" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="C10" s="4" t="s">
         <v>13</v>
@@ -716,7 +716,7 @@
         <v>10</v>
       </c>
       <c r="F10" s="5" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
     </row>
     <row r="11" ht="30.0" customHeight="1">
@@ -724,7 +724,7 @@
         <v>7.0</v>
       </c>
       <c r="B11" s="5" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="C11" s="4" t="s">
         <v>18</v>
@@ -733,10 +733,10 @@
         <v>46313.0</v>
       </c>
       <c r="E11" s="7" t="s">
-        <v>19</v>
+        <v>10</v>
       </c>
       <c r="F11" s="5" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
     </row>
     <row r="12" ht="30.0" customHeight="1">
@@ -744,7 +744,7 @@
         <v>8.0</v>
       </c>
       <c r="B12" s="5" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="C12" s="4" t="s">
         <v>9</v>
@@ -756,7 +756,7 @@
         <v>10</v>
       </c>
       <c r="F12" s="5" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
     </row>
     <row r="13" ht="30.0" customHeight="1">
@@ -764,7 +764,7 @@
         <v>9.0</v>
       </c>
       <c r="B13" s="5" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="C13" s="4" t="s">
         <v>18</v>
@@ -772,11 +772,11 @@
       <c r="D13" s="6">
         <v>46314.0</v>
       </c>
-      <c r="E13" s="4" t="s">
-        <v>30</v>
+      <c r="E13" s="7" t="s">
+        <v>10</v>
       </c>
       <c r="F13" s="5" t="s">
-        <v>31</v>
+        <v>29</v>
       </c>
     </row>
     <row r="14" ht="30.0" customHeight="1">
@@ -784,7 +784,7 @@
         <v>10.0</v>
       </c>
       <c r="B14" s="5" t="s">
-        <v>32</v>
+        <v>30</v>
       </c>
       <c r="C14" s="4" t="s">
         <v>9</v>
@@ -792,11 +792,11 @@
       <c r="D14" s="6">
         <v>46315.0</v>
       </c>
-      <c r="E14" s="4" t="s">
-        <v>30</v>
+      <c r="E14" s="7" t="s">
+        <v>10</v>
       </c>
       <c r="F14" s="5" t="s">
-        <v>33</v>
+        <v>31</v>
       </c>
     </row>
     <row r="15" ht="30.0" customHeight="1">
@@ -804,19 +804,19 @@
         <v>11.0</v>
       </c>
       <c r="B15" s="5" t="s">
-        <v>34</v>
+        <v>32</v>
       </c>
       <c r="C15" s="4" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="D15" s="6">
         <v>46317.0</v>
       </c>
-      <c r="E15" s="4" t="s">
-        <v>30</v>
+      <c r="E15" s="7" t="s">
+        <v>34</v>
       </c>
       <c r="F15" s="5" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
     </row>
     <row r="16" ht="30.0" customHeight="1">
@@ -824,19 +824,19 @@
         <v>12.0</v>
       </c>
       <c r="B16" s="5" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="C16" s="4" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="D16" s="6">
         <v>46318.0</v>
       </c>
-      <c r="E16" s="4" t="s">
-        <v>30</v>
+      <c r="E16" s="7" t="s">
+        <v>34</v>
       </c>
       <c r="F16" s="5" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
     </row>
     <row r="17" ht="30.0" customHeight="1">
@@ -844,7 +844,7 @@
         <v>13.0</v>
       </c>
       <c r="B17" s="5" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="C17" s="4" t="s">
         <v>9</v>
@@ -853,7 +853,7 @@
         <v>46318.0</v>
       </c>
       <c r="E17" s="4" t="s">
-        <v>30</v>
+        <v>39</v>
       </c>
       <c r="F17" s="5" t="s">
         <v>40</v>
@@ -867,13 +867,13 @@
         <v>41</v>
       </c>
       <c r="C18" s="4" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="D18" s="6">
         <v>46318.0</v>
       </c>
       <c r="E18" s="4" t="s">
-        <v>30</v>
+        <v>39</v>
       </c>
       <c r="F18" s="5" t="s">
         <v>42</v>
@@ -887,13 +887,13 @@
         <v>43</v>
       </c>
       <c r="C19" s="4" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="D19" s="6">
         <v>46319.0</v>
       </c>
       <c r="E19" s="4" t="s">
-        <v>30</v>
+        <v>39</v>
       </c>
       <c r="F19" s="5" t="s">
         <v>44</v>
@@ -913,7 +913,7 @@
         <v>46319.0</v>
       </c>
       <c r="E20" s="4" t="s">
-        <v>30</v>
+        <v>39</v>
       </c>
       <c r="F20" s="5" t="s">
         <v>46</v>
@@ -933,7 +933,7 @@
         <v>46320.0</v>
       </c>
       <c r="E21" s="4" t="s">
-        <v>30</v>
+        <v>39</v>
       </c>
       <c r="F21" s="5" t="s">
         <v>48</v>
@@ -947,11 +947,11 @@
     </row>
     <row r="24" ht="15.75" customHeight="1">
       <c r="B24" s="9" t="s">
-        <v>30</v>
+        <v>39</v>
       </c>
       <c r="C24" s="10">
         <f t="shared" ref="C24:C27" si="1">COUNTIF($E$5:$E$21,B24)</f>
-        <v>9</v>
+        <v>5</v>
       </c>
     </row>
     <row r="25" ht="15.75" customHeight="1">
@@ -965,7 +965,7 @@
     </row>
     <row r="26" ht="15.75" customHeight="1">
       <c r="B26" s="9" t="s">
-        <v>19</v>
+        <v>34</v>
       </c>
       <c r="C26" s="10">
         <f t="shared" si="1"/>
@@ -978,7 +978,7 @@
       </c>
       <c r="C27" s="10">
         <f t="shared" si="1"/>
-        <v>6</v>
+        <v>10</v>
       </c>
     </row>
     <row r="28" ht="15.75" customHeight="1">
@@ -996,7 +996,7 @@
       </c>
       <c r="C29" s="13">
         <f>IF(C28=0,0,C27/C28)</f>
-        <v>0.3529411765</v>
+        <v>0.5882352941</v>
       </c>
     </row>
     <row r="30" ht="15.75" customHeight="1"/>
@@ -2008,7 +2008,7 @@
   </conditionalFormatting>
   <dataValidations>
     <dataValidation type="list" allowBlank="1" sqref="E5:E21">
-      <formula1>"Por hacer,En progreso,En revisión,Listo"</formula1>
+      <formula1>"Por hacer,En progreso,En revisión,Listo,Incompleto"</formula1>
     </dataValidation>
   </dataValidations>
   <printOptions/>

</xml_diff>